<commit_message>
Before altitude, should still be 65.8%
</commit_message>
<xml_diff>
--- a/2026-06-27.xlsx
+++ b/2026-06-27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\Glicko-2, Etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE102F42-4CCB-4156-ABA2-83FBDE2354FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D1943E-0940-4674-911C-58F304B048FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="66">
   <si>
     <t>Red Corner</t>
   </si>
@@ -139,9 +139,6 @@
     <t>Bantamweight</t>
   </si>
   <si>
-    <t>Model</t>
-  </si>
-  <si>
     <t>Glicko-2</t>
   </si>
   <si>
@@ -214,7 +211,13 @@
     <t>-200</t>
   </si>
   <si>
-    <t>Blend</t>
+    <t>Final Pick</t>
+  </si>
+  <si>
+    <t>Blended Model</t>
+  </si>
+  <si>
+    <t>Raw Model</t>
   </si>
 </sst>
 </file>
@@ -268,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -300,11 +303,76 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -315,13 +383,42 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -624,710 +721,674 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5703125" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5703125" customWidth="1"/>
+    <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="D1" s="6"/>
-      <c r="E1" s="5" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="F1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="8"/>
+      <c r="H1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="5" t="s">
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="8"/>
+      <c r="Q1" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="S1" s="5"/>
+      <c r="R1" s="8"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="P2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="Q2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="R2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="12">
+        <v>0.60601742899335065</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="3">
         <v>0.52189291564157836</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="3">
+      <c r="K3" s="3">
         <v>0.51980099441760885</v>
       </c>
-      <c r="I3" s="3">
+      <c r="L3" s="3">
         <v>0.21138185740998641</v>
       </c>
-      <c r="J3" s="3">
+      <c r="M3" s="3">
         <v>0.51980099441760885</v>
       </c>
-      <c r="K3" s="3">
+      <c r="N3" s="12">
         <v>0.26881714817240482</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="3">
-        <v>0.60601742899335065</v>
-      </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="12">
+        <v>0.60458861993405388</v>
+      </c>
+      <c r="Q3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="3">
-        <v>0.60458861993405388</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="S3" s="2" t="s">
+      <c r="R3" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="12">
+        <v>0.61002431210091312</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="3">
         <v>0.66957149920152259</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="3">
+      <c r="K4" s="3">
         <v>0.56522345368794613</v>
       </c>
-      <c r="I4" s="3">
+      <c r="L4" s="3">
         <v>0.56522345368794613</v>
       </c>
-      <c r="J4" s="3">
+      <c r="M4" s="3">
         <v>0.38602955999950489</v>
       </c>
-      <c r="K4" s="3">
+      <c r="N4" s="12">
         <v>4.8746986312548972E-2</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="3">
-        <v>0.61002431210091312</v>
-      </c>
-      <c r="P4" s="2" t="s">
+      <c r="P4" s="12">
+        <v>0.54732038663722149</v>
+      </c>
+      <c r="Q4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="Q4" s="3">
-        <v>0.54732038663722149</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="S4" s="2" t="s">
+      <c r="R4" s="15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="12">
+        <v>0.60670082680913917</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="3">
         <v>0.50543782296166417</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="3">
+      <c r="K5" s="3">
         <v>0.42280686820599389</v>
       </c>
-      <c r="I5" s="3">
+      <c r="L5" s="3">
         <v>0.42280686820599389</v>
       </c>
-      <c r="J5" s="3">
+      <c r="M5" s="3">
         <v>0.21045311784064591</v>
       </c>
-      <c r="K5" s="3">
+      <c r="N5" s="12">
         <v>0.36674001395336009</v>
       </c>
-      <c r="L5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="O5" s="3">
-        <v>0.60670082680913917</v>
-      </c>
-      <c r="P5" s="2" t="s">
+      <c r="O5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="P5" s="12">
         <v>0.72044640970692841</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="Q5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="S5" s="2" t="s">
+      <c r="R5" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="12">
+        <v>0.73305617349770713</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="3">
         <v>0.75451286349842606</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="3">
+      <c r="K6" s="3">
         <v>0.55415822359232592</v>
       </c>
-      <c r="I6" s="3">
+      <c r="L6" s="3">
         <v>0.55415822359232592</v>
       </c>
-      <c r="J6" s="3">
+      <c r="M6" s="3">
         <v>6.6158259444694931E-2</v>
       </c>
-      <c r="K6" s="3">
+      <c r="N6" s="12">
         <v>0.37968351696297908</v>
       </c>
-      <c r="L6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="N6" s="2" t="s">
+      <c r="O6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="3">
-        <v>0.73305617349770713</v>
-      </c>
-      <c r="P6" s="2" t="s">
+      <c r="P6" s="12">
+        <v>0.63760165463337459</v>
+      </c>
+      <c r="Q6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="Q6" s="3">
-        <v>0.63760165463337459</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="S6" s="2" t="s">
+      <c r="R6" s="15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="12">
+        <v>0.63907577983265651</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="3">
         <v>0.68313527612609992</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="3">
+      <c r="K7" s="3">
         <v>0.38736898552586518</v>
       </c>
-      <c r="I7" s="3">
+      <c r="L7" s="3">
         <v>0.25521724663986478</v>
       </c>
-      <c r="J7" s="3">
+      <c r="M7" s="3">
         <v>0.38736898552586518</v>
       </c>
-      <c r="K7" s="3">
+      <c r="N7" s="12">
         <v>0.35741376783426998</v>
       </c>
-      <c r="L7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="N7" s="2" t="s">
+      <c r="O7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="O7" s="3">
-        <v>0.63907577983265651</v>
-      </c>
-      <c r="P7" s="2" t="s">
+      <c r="P7" s="12">
+        <v>0.60646421362230318</v>
+      </c>
+      <c r="Q7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="Q7" s="3">
-        <v>0.60646421362230318</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="S7" s="2" t="s">
+      <c r="R7" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0.58661624915147503</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="3">
+      <c r="I8" s="3">
         <v>0.52519218407540535</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="H8" s="3">
-        <v>0.5979158963468183</v>
-      </c>
-      <c r="I8" s="3">
-        <v>0.2819158469948409</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0.1201682566583408</v>
       </c>
       <c r="K8" s="3">
         <v>0.5979158963468183</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="N8" s="2" t="s">
+      <c r="L8" s="3">
+        <v>0.2819158469948409</v>
+      </c>
+      <c r="M8" s="3">
+        <v>0.1201682566583408</v>
+      </c>
+      <c r="N8" s="12">
+        <v>0.5979158963468183</v>
+      </c>
+      <c r="O8" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="O8" s="3">
-        <v>0.58661624915147503</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q8" s="3">
+      <c r="P8" s="12">
         <v>0.50302646258224548</v>
       </c>
-      <c r="R8" s="2" t="s">
+      <c r="Q8" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="S8" s="2" t="s">
+      <c r="R8" s="15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="12">
+        <v>0.66653276005944706</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="3">
         <v>0.73973677769637292</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="H9" s="3">
-        <v>0.50185982393426898</v>
-      </c>
-      <c r="I9" s="3">
-        <v>0.2365283347784381</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0.26161184128729292</v>
       </c>
       <c r="K9" s="3">
         <v>0.50185982393426898</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="N9" s="2" t="s">
+      <c r="L9" s="3">
+        <v>0.2365283347784381</v>
+      </c>
+      <c r="M9" s="3">
+        <v>0.26161184128729292</v>
+      </c>
+      <c r="N9" s="12">
+        <v>0.50185982393426898</v>
+      </c>
+      <c r="O9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="O9" s="3">
-        <v>0.66653276005944706</v>
-      </c>
-      <c r="P9" s="2" t="s">
+      <c r="P9" s="12">
+        <v>0.68750343162428518</v>
+      </c>
+      <c r="Q9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="Q9" s="3">
-        <v>0.68750343162428518</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S9" s="2" t="s">
+      <c r="R9" s="15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="12">
+        <v>0.51918696076230797</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="3">
         <v>0.60727156492295187</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="3">
+      <c r="K10" s="3">
         <v>0.47770470224071859</v>
       </c>
-      <c r="I10" s="3">
+      <c r="L10" s="3">
         <v>0.47770470224071859</v>
       </c>
-      <c r="J10" s="3">
+      <c r="M10" s="3">
         <v>0.39563958808490268</v>
       </c>
-      <c r="K10" s="3">
+      <c r="N10" s="12">
         <v>0.1266557096743787</v>
       </c>
-      <c r="L10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="N10" s="2" t="s">
+      <c r="O10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="O10" s="3">
-        <v>0.51918696076230797</v>
-      </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="12">
+        <v>0.6645065560009189</v>
+      </c>
+      <c r="Q10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="Q10" s="3">
-        <v>0.6645065560009189</v>
-      </c>
-      <c r="R10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="S10" s="2" t="s">
+      <c r="R10" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="12">
+        <v>0.60996337476194262</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="3">
         <v>0.59498711870039145</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="3">
+      <c r="K11" s="3">
         <v>0.51533246390173004</v>
       </c>
-      <c r="I11" s="3">
+      <c r="L11" s="3">
         <v>0.27342142353977089</v>
       </c>
-      <c r="J11" s="3">
+      <c r="M11" s="3">
         <v>0.51533246390173004</v>
       </c>
-      <c r="K11" s="3">
+      <c r="N11" s="12">
         <v>0.21124611255849901</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="N11" s="2" t="s">
+      <c r="O11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="O11" s="3">
-        <v>0.60996337476194262</v>
-      </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" s="12">
+        <v>0.62211224869346138</v>
+      </c>
+      <c r="Q11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="Q11" s="3">
-        <v>0.62211224869346138</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="S11" s="2" t="s">
+      <c r="R11" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="12">
+        <v>0.59715165162995332</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="3">
         <v>0.62027103611953671</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="3">
+      <c r="K12" s="3">
         <v>0.51906027486062123</v>
       </c>
-      <c r="I12" s="3">
+      <c r="L12" s="3">
         <v>0.51906027486062123</v>
       </c>
-      <c r="J12" s="3">
+      <c r="M12" s="3">
         <v>0.1943946314831034</v>
       </c>
-      <c r="K12" s="3">
+      <c r="N12" s="12">
         <v>0.28654509365627551</v>
       </c>
-      <c r="L12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N12" s="2" t="s">
+      <c r="O12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="O12" s="3">
-        <v>0.59715165162995332</v>
-      </c>
-      <c r="P12" s="2" t="s">
+      <c r="P12" s="12">
+        <v>0.65599422095448756</v>
+      </c>
+      <c r="Q12" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="Q12" s="3">
-        <v>0.65599422095448756</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="S12" s="3" t="s">
+      <c r="R12" s="12" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="E1:K1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:N1"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="Q1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added raw elevation in feet input
</commit_message>
<xml_diff>
--- a/2026-06-27.xlsx
+++ b/2026-06-27.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\Glicko-2, Etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D1943E-0940-4674-911C-58F304B048FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4ED09F-1B3C-49D3-A6D1-E82A42A8B8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Predictions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="68">
   <si>
     <t>Red Corner</t>
   </si>
@@ -157,60 +157,9 @@
     <t>Model %</t>
   </si>
   <si>
-    <t>-142</t>
-  </si>
-  <si>
-    <t>+120</t>
-  </si>
-  <si>
-    <t>-300</t>
-  </si>
-  <si>
     <t>+250</t>
   </si>
   <si>
-    <t>-160</t>
-  </si>
-  <si>
-    <t>+140</t>
-  </si>
-  <si>
-    <t>-400</t>
-  </si>
-  <si>
-    <t>+330</t>
-  </si>
-  <si>
-    <t>-190</t>
-  </si>
-  <si>
-    <t>+165</t>
-  </si>
-  <si>
-    <t>-500</t>
-  </si>
-  <si>
-    <t>+385</t>
-  </si>
-  <si>
-    <t>-250</t>
-  </si>
-  <si>
-    <t>+210</t>
-  </si>
-  <si>
-    <t>+130</t>
-  </si>
-  <si>
-    <t>-150</t>
-  </si>
-  <si>
-    <t>+170</t>
-  </si>
-  <si>
-    <t>-200</t>
-  </si>
-  <si>
     <t>Final Pick</t>
   </si>
   <si>
@@ -218,6 +167,63 @@
   </si>
   <si>
     <t>Raw Model</t>
+  </si>
+  <si>
+    <t>-117</t>
+  </si>
+  <si>
+    <t>+100</t>
+  </si>
+  <si>
+    <t>-346</t>
+  </si>
+  <si>
+    <t>+281</t>
+  </si>
+  <si>
+    <t>-238</t>
+  </si>
+  <si>
+    <t>+199</t>
+  </si>
+  <si>
+    <t>-236</t>
+  </si>
+  <si>
+    <t>+198</t>
+  </si>
+  <si>
+    <t>-304</t>
+  </si>
+  <si>
+    <t>-137</t>
+  </si>
+  <si>
+    <t>+118</t>
+  </si>
+  <si>
+    <t>-525</t>
+  </si>
+  <si>
+    <t>+404</t>
+  </si>
+  <si>
+    <t>-217</t>
+  </si>
+  <si>
+    <t>+183</t>
+  </si>
+  <si>
+    <t>+143</t>
+  </si>
+  <si>
+    <t>-168</t>
+  </si>
+  <si>
+    <t>+138</t>
+  </si>
+  <si>
+    <t>-162</t>
   </si>
 </sst>
 </file>
@@ -271,7 +277,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -304,19 +310,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -372,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -383,41 +376,35 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -745,27 +732,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="F1" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="8"/>
-      <c r="H1" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="7" t="s">
+      <c r="F1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="12"/>
+      <c r="H1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="7" t="s">
+      <c r="P1" s="12"/>
+      <c r="Q1" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="R1" s="8"/>
+      <c r="R1" s="12"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -780,17 +767,17 @@
       <c r="D2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>63</v>
+      <c r="H2" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>4</v>
@@ -807,19 +794,19 @@
       <c r="M2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="R2" s="9" t="s">
         <v>5</v>
       </c>
     </row>
@@ -828,54 +815,54 @@
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="12">
-        <v>0.60601742899335065</v>
-      </c>
-      <c r="H3" s="11" t="s">
+      <c r="G3" s="7">
+        <v>0.5911791319827927</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="I3" s="3">
-        <v>0.52189291564157836</v>
+        <v>0.53661163391721933</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="K3" s="3">
-        <v>0.51980099441760885</v>
+        <v>0.57245245780198561</v>
       </c>
       <c r="L3" s="3">
-        <v>0.21138185740998641</v>
+        <v>0.19986417358748501</v>
       </c>
       <c r="M3" s="3">
-        <v>0.51980099441760885</v>
-      </c>
-      <c r="N3" s="12">
-        <v>0.26881714817240482</v>
-      </c>
-      <c r="O3" s="11" t="s">
+        <v>0.57245245780198561</v>
+      </c>
+      <c r="N3" s="7">
+        <v>0.2276833686105294</v>
+      </c>
+      <c r="O3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="P3" s="12">
+      <c r="P3" s="7">
         <v>0.60458861993405388</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="Q3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="R3" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -884,54 +871,54 @@
         <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="12">
-        <v>0.61002431210091312</v>
-      </c>
-      <c r="H4" s="11" t="s">
+      <c r="G4" s="7">
+        <v>0.56286831321049358</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="I4" s="3">
-        <v>0.66957149920152259</v>
+        <v>0.66111793999037216</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="K4" s="3">
-        <v>0.56522345368794613</v>
+        <v>0.49490648124665387</v>
       </c>
       <c r="L4" s="3">
-        <v>0.56522345368794613</v>
+        <v>0.49490648124665387</v>
       </c>
       <c r="M4" s="3">
-        <v>0.38602955999950489</v>
-      </c>
-      <c r="N4" s="12">
-        <v>4.8746986312548972E-2</v>
-      </c>
-      <c r="O4" s="11" t="s">
+        <v>0.44030278530984079</v>
+      </c>
+      <c r="N4" s="7">
+        <v>6.4790733443505236E-2</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P4" s="12">
+      <c r="P4" s="7">
         <v>0.54732038663722149</v>
       </c>
-      <c r="Q4" s="11" t="s">
+      <c r="Q4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="R4" s="15" t="s">
+      <c r="R4" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -940,54 +927,54 @@
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="12">
-        <v>0.60670082680913917</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>19</v>
+      <c r="G5" s="7">
+        <v>0.6548267133663902</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I5" s="3">
-        <v>0.50543782296166417</v>
+        <v>0.51301881869598998</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K5" s="3">
-        <v>0.42280686820599389</v>
+        <v>0.45256309562386809</v>
       </c>
       <c r="L5" s="3">
-        <v>0.42280686820599389</v>
+        <v>0.32849666928331211</v>
       </c>
       <c r="M5" s="3">
-        <v>0.21045311784064591</v>
-      </c>
-      <c r="N5" s="12">
-        <v>0.36674001395336009</v>
-      </c>
-      <c r="O5" s="11" t="s">
+        <v>0.45256309562386809</v>
+      </c>
+      <c r="N5" s="7">
+        <v>0.21894023509281979</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="7">
         <v>0.72044640970692841</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="R5" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -996,54 +983,54 @@
         <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="12">
-        <v>0.73305617349770713</v>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="G6" s="7">
+        <v>0.76613500679650626</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>21</v>
       </c>
       <c r="I6" s="3">
-        <v>0.75451286349842606</v>
+        <v>0.72364790105069932</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="K6" s="3">
-        <v>0.55415822359232592</v>
+        <v>0.53793803186643319</v>
       </c>
       <c r="L6" s="3">
-        <v>0.55415822359232592</v>
+        <v>0.53793803186643319</v>
       </c>
       <c r="M6" s="3">
-        <v>6.6158259444694931E-2</v>
-      </c>
-      <c r="N6" s="12">
-        <v>0.37968351696297908</v>
-      </c>
-      <c r="O6" s="11" t="s">
+        <v>0.1013517617843914</v>
+      </c>
+      <c r="N6" s="7">
+        <v>0.3607102063491755</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="7">
         <v>0.63760165463337459</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="15" t="s">
+      <c r="R6" s="10" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1052,54 +1039,54 @@
         <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="12">
-        <v>0.63907577983265651</v>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="G7" s="7">
+        <v>0.59429042583285407</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>24</v>
       </c>
       <c r="I7" s="3">
-        <v>0.68313527612609992</v>
+        <v>0.6626337251318638</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="K7" s="3">
-        <v>0.38736898552586518</v>
+        <v>0.47462664869620502</v>
       </c>
       <c r="L7" s="3">
-        <v>0.25521724663986478</v>
+        <v>0.24649257687848519</v>
       </c>
       <c r="M7" s="3">
-        <v>0.38736898552586518</v>
-      </c>
-      <c r="N7" s="12">
-        <v>0.35741376783426998</v>
-      </c>
-      <c r="O7" s="11" t="s">
+        <v>0.47462664869620502</v>
+      </c>
+      <c r="N7" s="7">
+        <v>0.27888077442530979</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="7">
         <v>0.60646421362230318</v>
       </c>
-      <c r="Q7" s="11" t="s">
+      <c r="Q7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="R7" s="15" t="s">
+      <c r="R7" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1108,54 +1095,54 @@
         <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="12">
-        <v>0.58661624915147503</v>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="G8" s="7">
+        <v>0.61664921141142215</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0.53047520201461584</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="3">
+        <v>0.66834112177314087</v>
+      </c>
+      <c r="L8" s="3">
+        <v>0.19995082795024949</v>
+      </c>
+      <c r="M8" s="3">
+        <v>0.66834112177314087</v>
+      </c>
+      <c r="N8" s="7">
+        <v>0.13170805027660959</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="7">
+        <v>0.50302646258224548</v>
+      </c>
+      <c r="Q8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="3">
-        <v>0.52519218407540535</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="3">
-        <v>0.5979158963468183</v>
-      </c>
-      <c r="L8" s="3">
-        <v>0.2819158469948409</v>
-      </c>
-      <c r="M8" s="3">
-        <v>0.1201682566583408</v>
-      </c>
-      <c r="N8" s="12">
-        <v>0.5979158963468183</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="12">
-        <v>0.50302646258224548</v>
-      </c>
-      <c r="Q8" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="R8" s="15" t="s">
+      <c r="R8" s="10" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1164,54 +1151,54 @@
         <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="12">
-        <v>0.66653276005944706</v>
-      </c>
-      <c r="H9" s="11" t="s">
+      <c r="G9" s="7">
+        <v>0.69875432793535353</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>28</v>
       </c>
       <c r="I9" s="3">
-        <v>0.73973677769637292</v>
+        <v>0.75808569794957281</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="K9" s="3">
-        <v>0.50185982393426898</v>
+        <v>0.46199971696846809</v>
       </c>
       <c r="L9" s="3">
-        <v>0.2365283347784381</v>
+        <v>0.2215737121375716</v>
       </c>
       <c r="M9" s="3">
-        <v>0.26161184128729292</v>
-      </c>
-      <c r="N9" s="12">
-        <v>0.50185982393426898</v>
-      </c>
-      <c r="O9" s="11" t="s">
+        <v>0.31642657089396031</v>
+      </c>
+      <c r="N9" s="7">
+        <v>0.46199971696846809</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="7">
         <v>0.68750343162428518</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="Q9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="R9" s="15" t="s">
+      <c r="R9" s="10" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1220,54 +1207,54 @@
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="7">
+        <v>0.57453969876025912</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="12">
-        <v>0.51918696076230797</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>31</v>
-      </c>
       <c r="I10" s="3">
-        <v>0.60727156492295187</v>
+        <v>0.54498735177779922</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="K10" s="3">
-        <v>0.47770470224071859</v>
+        <v>0.45930752885018677</v>
       </c>
       <c r="L10" s="3">
-        <v>0.47770470224071859</v>
+        <v>0.45930752885018677</v>
       </c>
       <c r="M10" s="3">
-        <v>0.39563958808490268</v>
-      </c>
-      <c r="N10" s="12">
-        <v>0.1266557096743787</v>
-      </c>
-      <c r="O10" s="11" t="s">
+        <v>0.41001964346457243</v>
+      </c>
+      <c r="N10" s="7">
+        <v>0.1306728276852408</v>
+      </c>
+      <c r="O10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="P10" s="12">
+      <c r="P10" s="7">
         <v>0.6645065560009189</v>
       </c>
-      <c r="Q10" s="11" t="s">
+      <c r="Q10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="R10" s="15" t="s">
+      <c r="R10" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1276,54 +1263,54 @@
         <v>33</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="12">
-        <v>0.60996337476194262</v>
-      </c>
-      <c r="H11" s="11" t="s">
+      <c r="G11" s="7">
+        <v>0.56909449671137691</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>34</v>
       </c>
       <c r="I11" s="3">
-        <v>0.59498711870039145</v>
+        <v>0.58649946988423407</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="K11" s="3">
-        <v>0.51533246390173004</v>
+        <v>0.52455958075329112</v>
       </c>
       <c r="L11" s="3">
-        <v>0.27342142353977089</v>
+        <v>0.29621246462700951</v>
       </c>
       <c r="M11" s="3">
-        <v>0.51533246390173004</v>
-      </c>
-      <c r="N11" s="12">
-        <v>0.21124611255849901</v>
-      </c>
-      <c r="O11" s="11" t="s">
+        <v>0.52455958075329112</v>
+      </c>
+      <c r="N11" s="7">
+        <v>0.17922795461969929</v>
+      </c>
+      <c r="O11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="7">
         <v>0.62211224869346138</v>
       </c>
-      <c r="Q11" s="11" t="s">
+      <c r="Q11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="R11" s="15" t="s">
+      <c r="R11" s="10" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1332,54 +1319,54 @@
         <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G12" s="12">
-        <v>0.59715165162995332</v>
-      </c>
-      <c r="H12" s="11" t="s">
+      <c r="G12" s="7">
+        <v>0.59476912470453525</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>37</v>
       </c>
       <c r="I12" s="3">
-        <v>0.62027103611953671</v>
+        <v>0.59508674558334707</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="K12" s="3">
-        <v>0.51906027486062123</v>
+        <v>0.54226238691743189</v>
       </c>
       <c r="L12" s="3">
-        <v>0.51906027486062123</v>
+        <v>0.54226238691743189</v>
       </c>
       <c r="M12" s="3">
-        <v>0.1943946314831034</v>
-      </c>
-      <c r="N12" s="12">
-        <v>0.28654509365627551</v>
-      </c>
-      <c r="O12" s="11" t="s">
+        <v>0.22407796546715619</v>
+      </c>
+      <c r="N12" s="7">
+        <v>0.233659647615412</v>
+      </c>
+      <c r="O12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="7">
         <v>0.65599422095448756</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="R12" s="12" t="s">
+      <c r="R12" s="7" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>